<commit_message>
Build runbook version 2.3 DOCX, PDF and sizing calculator
Co-authored-by: ravislr-beep <ravislr-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runbook/out/Pega_26_Sizing_Calculator.xlsx
+++ b/runbook/out/Pega_26_Sizing_Calculator.xlsx
@@ -549,7 +549,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>AKS zone headroom of 1.5 and one surge node: this design (runbook Section 4.6).</t>
+          <t>AKS zone headroom of 1.5 (PERF, PREPROD, PROD) or 1.0 (DEV, SIT, UAT) and one surge node: this design (runbook Section 4.6).</t>
         </is>
       </c>
     </row>
@@ -1451,12 +1451,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1472,6 +1473,11 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>NP1 Pega pool</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -1485,7 +1491,10 @@
       <c r="B2" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Sum of tier HPA maximums</t>
         </is>
@@ -1500,7 +1509,10 @@
       <c r="B3" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Chart default 3</t>
         </is>
@@ -1515,7 +1527,10 @@
       <c r="B4" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Chart default 12Gi</t>
         </is>
@@ -1530,7 +1545,10 @@
       <c r="B5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>kubectl describe node; after system reservations</t>
         </is>
@@ -1545,9 +1563,30 @@
       <c r="B6" s="6" t="n">
         <v>58</v>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>kubectl describe node</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Zone headroom factor</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>1.5 for PERF, PREPROD and PROD so two zones carry the peak; 1.0 for DEV, SIT and UAT (Section 4.6)</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1600,11 @@
         <f>MIN(ROUNDDOWN(B5/B3,0),ROUNDDOWN(B6/B4,0))</f>
         <v/>
       </c>
-      <c r="C8" s="7" t="inlineStr"/>
+      <c r="C8" s="8">
+        <f>MIN(ROUNDDOWN(C5/C3,0),ROUNDDOWN(C6/C4,0))</f>
+        <v/>
+      </c>
+      <c r="D8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -1573,7 +1616,11 @@
         <f>ROUNDUP(B2/B8,0)</f>
         <v/>
       </c>
-      <c r="C9" s="7" t="inlineStr"/>
+      <c r="C9" s="8">
+        <f>ROUNDUP(C2/C8,0)</f>
+        <v/>
+      </c>
+      <c r="D9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1582,12 +1629,16 @@
         </is>
       </c>
       <c r="B10" s="8">
-        <f>CEILING(ROUNDUP(B9*1.5,0)+1,3)</f>
-        <v/>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>x 1.5 so two zones carry the peak; +1 surge node; multiple of 3</t>
+        <f>CEILING(ROUNDUP(B9*B7,0)+1,3)</f>
+        <v/>
+      </c>
+      <c r="C10" s="8">
+        <f>CEILING(ROUNDUP(C9*C7,0)+1,3)</f>
+        <v/>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>x headroom factor; +1 surge node; multiple of 3</t>
         </is>
       </c>
     </row>

</xml_diff>